<commit_message>
agregado de munita de reunion y toma de asistencia
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gcasas\CopaRobotica2026\documentacion\generada\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="alumnos" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Asistencia" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="alumnos" sheetId="1" r:id="rId1"/>
+    <sheet name="Asistencia" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -21,504 +25,504 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="198">
-  <si>
-    <t xml:space="preserve">Alumnos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">º</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">apellido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nombres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fecha de envio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">correo electronoica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fecha de nacimiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">curso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">especialidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">obs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">grupo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Andrada Bascope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Victoria Abril </t>
-  </si>
-  <si>
-    <t xml:space="preserve">tory.and.bas@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avionica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ok para cargar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIR-321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cantelli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">chucusea Quiroga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zaira Ruth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">quiroruth1@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSI-258</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Casas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Farías Ruiz </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paloma Marianella</t>
-  </si>
-  <si>
-    <t xml:space="preserve">palofariasruiz@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13/04/2011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NQG-987</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juncal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demian Ignacio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">juncaldemian12@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16/04/2010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcaraz, Juncal, Lucero, Lujan, Manrique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lujan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiago Gabriel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thiaguitolujan09@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">joaquin alcaraz, juncal demian, lujan thiago, lucero valentin, Tahiel manrique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PBM-741</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Da Costa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luna Serrano </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benicio valentin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">benicio.luna11@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maidana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin Nahuel</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> kevinmaidana315@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10/08/2009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JKQ-448</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Molinero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mateo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mateoprado2701@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ravanelli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ivan Manuel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ivanravanelli912@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XNN-744</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cuenca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trinidad Sanabria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carlos Leonel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c.l.t.s.acad@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31/10/2007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matías Hernan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matruia81@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcaraz</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="196">
+  <si>
+    <t>Alumnos</t>
+  </si>
+  <si>
+    <t>º</t>
+  </si>
+  <si>
+    <t>nro</t>
+  </si>
+  <si>
+    <t>apellido</t>
+  </si>
+  <si>
+    <t>nombres</t>
+  </si>
+  <si>
+    <t>dni</t>
+  </si>
+  <si>
+    <t>fecha de envio</t>
+  </si>
+  <si>
+    <t>correo electronoica</t>
+  </si>
+  <si>
+    <t>fecha de nacimiento</t>
+  </si>
+  <si>
+    <t>curso</t>
+  </si>
+  <si>
+    <t>especialidad</t>
+  </si>
+  <si>
+    <t>obs</t>
+  </si>
+  <si>
+    <t>grupo</t>
+  </si>
+  <si>
+    <t>Docente</t>
+  </si>
+  <si>
+    <t>Andrada Bascope</t>
+  </si>
+  <si>
+    <t>Victoria Abril </t>
+  </si>
+  <si>
+    <t>tory.and.bas@gmail.com</t>
+  </si>
+  <si>
+    <t>4B</t>
+  </si>
+  <si>
+    <t>avionica</t>
+  </si>
+  <si>
+    <t>ok para cargar</t>
+  </si>
+  <si>
+    <t>SIR-321</t>
+  </si>
+  <si>
+    <t>Cantelli</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>chucusea Quiroga</t>
+  </si>
+  <si>
+    <t>Zaira Ruth</t>
+  </si>
+  <si>
+    <t>quiroruth1@gmail.com</t>
+  </si>
+  <si>
+    <t>BSI-258</t>
+  </si>
+  <si>
+    <t>Casas</t>
+  </si>
+  <si>
+    <t>Farías Ruiz </t>
+  </si>
+  <si>
+    <t>Paloma Marianella</t>
+  </si>
+  <si>
+    <t>palofariasruiz@gmail.com</t>
+  </si>
+  <si>
+    <t>13/04/2011</t>
+  </si>
+  <si>
+    <t>NQG-987</t>
+  </si>
+  <si>
+    <t>Pages</t>
+  </si>
+  <si>
+    <t>Juncal</t>
+  </si>
+  <si>
+    <t>Demian Ignacio</t>
+  </si>
+  <si>
+    <t>juncaldemian12@gmail.com</t>
+  </si>
+  <si>
+    <t>16/04/2010</t>
+  </si>
+  <si>
+    <t>5A</t>
+  </si>
+  <si>
+    <t>Alcaraz, Juncal, Lucero, Lujan, Manrique</t>
+  </si>
+  <si>
+    <t>Lujan</t>
+  </si>
+  <si>
+    <t>Thiago Gabriel</t>
+  </si>
+  <si>
+    <t>thiaguitolujan09@gmail.com</t>
+  </si>
+  <si>
+    <t>joaquin alcaraz, juncal demian, lujan thiago, lucero valentin, Tahiel manrique</t>
+  </si>
+  <si>
+    <t>PBM-741</t>
+  </si>
+  <si>
+    <t>Da Costa</t>
+  </si>
+  <si>
+    <t>Luna Serrano </t>
+  </si>
+  <si>
+    <t>Benicio valentin</t>
+  </si>
+  <si>
+    <t>benicio.luna11@gmail.com</t>
+  </si>
+  <si>
+    <t>Maidana</t>
+  </si>
+  <si>
+    <t>Kevin Nahuel</t>
+  </si>
+  <si>
+    <t> kevinmaidana315@gmail.com</t>
+  </si>
+  <si>
+    <t>10/08/2009</t>
+  </si>
+  <si>
+    <t>5B</t>
+  </si>
+  <si>
+    <t>JKQ-448</t>
+  </si>
+  <si>
+    <t>Molinero</t>
+  </si>
+  <si>
+    <t>Prado</t>
+  </si>
+  <si>
+    <t>Mateo</t>
+  </si>
+  <si>
+    <t>mateoprado2701@gmail.com</t>
+  </si>
+  <si>
+    <t>Ravanelli</t>
+  </si>
+  <si>
+    <t>Ivan Manuel</t>
+  </si>
+  <si>
+    <t>ivanravanelli912@gmail.com</t>
+  </si>
+  <si>
+    <t>XNN-744</t>
+  </si>
+  <si>
+    <t>Cuenca</t>
+  </si>
+  <si>
+    <t>Trinidad Sanabria</t>
+  </si>
+  <si>
+    <t>Carlos Leonel</t>
+  </si>
+  <si>
+    <t>c.l.t.s.acad@gmail.com</t>
+  </si>
+  <si>
+    <t>31/10/2007</t>
+  </si>
+  <si>
+    <t>7A</t>
+  </si>
+  <si>
+    <t>Matías Hernan</t>
+  </si>
+  <si>
+    <t>matruia81@gmail.com</t>
+  </si>
+  <si>
+    <t>Alcaraz</t>
   </si>
   <si>
     <t xml:space="preserve">Joaquín Leandro David </t>
   </si>
   <si>
-    <t xml:space="preserve">Ven09130814@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcaraz, Juncal, Lucero, Luján, Manrique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alegre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sofía Angélica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sofialegre58@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arredondo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facundo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arredondofacundo406@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07/05/2010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arredondo facundo, Ravanelli Iván, Prado Mateos, Palermo Alejo, Martinez fabrizio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carrizo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiziano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tizianoinac23@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cetera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ulises Nicolás</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ulimirage3@gmail.com</t>
+    <t>Ven09130814@gmail.com</t>
+  </si>
+  <si>
+    <t>Alcaraz, Juncal, Lucero, Luján, Manrique</t>
+  </si>
+  <si>
+    <t>Alegre</t>
+  </si>
+  <si>
+    <t>Sofía Angélica</t>
+  </si>
+  <si>
+    <t>sofialegre58@gmail.com</t>
+  </si>
+  <si>
+    <t>6B</t>
+  </si>
+  <si>
+    <t>Arredondo</t>
+  </si>
+  <si>
+    <t>Facundo</t>
+  </si>
+  <si>
+    <t>arredondofacundo406@gmail.com</t>
+  </si>
+  <si>
+    <t>07/05/2010</t>
+  </si>
+  <si>
+    <t>Arredondo facundo, Ravanelli Iván, Prado Mateos, Palermo Alejo, Martinez fabrizio</t>
+  </si>
+  <si>
+    <t>Carrizo</t>
+  </si>
+  <si>
+    <t>Tiziano</t>
+  </si>
+  <si>
+    <t>tizianoinac23@gmail.com</t>
+  </si>
+  <si>
+    <t>Cetera</t>
+  </si>
+  <si>
+    <t>Ulises Nicolás</t>
+  </si>
+  <si>
+    <t>ulimirage3@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">Chiapparo </t>
   </si>
   <si>
-    <t xml:space="preserve">Tiago Benjamin</t>
+    <t>Tiago Benjamin</t>
   </si>
   <si>
     <t xml:space="preserve"> benjaniupi@gmail.com</t>
   </si>
   <si>
-    <t xml:space="preserve">16/09/2009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORREA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santino Jonas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">santycorreasd24@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20/10/2010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Farías Ruiz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candelaria Luisana </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giraldo Gonzalez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juan Diego</t>
-  </si>
-  <si>
-    <t xml:space="preserve">juandiegonzales1311@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13/11/2009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gómez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiago</t>
-  </si>
-  <si>
-    <t xml:space="preserve">punaxs31@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lemos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sophie Micaela</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sophielemos15@gmail.com </t>
-  </si>
-  <si>
-    <t xml:space="preserve">5/10/2010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lescano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mateobautistalescano123@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lucero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiago Valentín</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valentinluceroxd@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcaraz, Juncal, Lucero, Luján, Manrique </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MANRIQUE DI FLORIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tahiel Eliseo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tahiel.e.manrique@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcaraz, Juncal, Lucero, Lujan y Manrique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Martinez Ruiz Diaz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabrizio Juan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">martnezfabrizio84@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6/10/2009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Melin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Franco Ezequiel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">franmelin14@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22/06/2010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rodriguez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venus Yasmìn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ven09130814@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiseyra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Isabella Giuliana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">chidodejameempa@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18/11/2010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Videla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giuliana Abril</t>
-  </si>
-  <si>
-    <t xml:space="preserve">videlagiuliana4@gmail.com</t>
+    <t>16/09/2009</t>
+  </si>
+  <si>
+    <t>CORREA</t>
+  </si>
+  <si>
+    <t>Santino Jonas</t>
+  </si>
+  <si>
+    <t>santycorreasd24@gmail.com</t>
+  </si>
+  <si>
+    <t>20/10/2010</t>
+  </si>
+  <si>
+    <t>Farías Ruiz</t>
+  </si>
+  <si>
+    <t>Candelaria Luisana </t>
+  </si>
+  <si>
+    <t>Giraldo Gonzalez</t>
+  </si>
+  <si>
+    <t>Juan Diego</t>
+  </si>
+  <si>
+    <t>juandiegonzales1311@gmail.com</t>
+  </si>
+  <si>
+    <t>13/11/2009</t>
+  </si>
+  <si>
+    <t>Gómez</t>
+  </si>
+  <si>
+    <t>Thiago</t>
+  </si>
+  <si>
+    <t>punaxs31@gmail.com</t>
+  </si>
+  <si>
+    <t>Lemos</t>
+  </si>
+  <si>
+    <t>Sophie Micaela</t>
+  </si>
+  <si>
+    <t>sophielemos15@gmail.com </t>
+  </si>
+  <si>
+    <t>5/10/2010</t>
+  </si>
+  <si>
+    <t>Lescano</t>
+  </si>
+  <si>
+    <t>mateobautistalescano123@gmail.com</t>
+  </si>
+  <si>
+    <t>Lucero</t>
+  </si>
+  <si>
+    <t>Thiago Valentín</t>
+  </si>
+  <si>
+    <t>valentinluceroxd@gmail.com</t>
+  </si>
+  <si>
+    <t>Alcaraz, Juncal, Lucero, Luján, Manrique </t>
+  </si>
+  <si>
+    <t>MANRIQUE DI FLORIO</t>
+  </si>
+  <si>
+    <t>Tahiel Eliseo</t>
+  </si>
+  <si>
+    <t>tahiel.e.manrique@gmail.com</t>
+  </si>
+  <si>
+    <t>Alcaraz, Juncal, Lucero, Lujan y Manrique</t>
+  </si>
+  <si>
+    <t>Martinez Ruiz Diaz</t>
+  </si>
+  <si>
+    <t>Fabrizio Juan</t>
+  </si>
+  <si>
+    <t>martnezfabrizio84@gmail.com</t>
+  </si>
+  <si>
+    <t>6/10/2009</t>
+  </si>
+  <si>
+    <t>Melin</t>
+  </si>
+  <si>
+    <t>Franco Ezequiel</t>
+  </si>
+  <si>
+    <t>franmelin14@gmail.com</t>
+  </si>
+  <si>
+    <t>22/06/2010</t>
+  </si>
+  <si>
+    <t>Rodriguez</t>
+  </si>
+  <si>
+    <t>Venus Yasmìn</t>
+  </si>
+  <si>
+    <t>ven09130814@gmail.com</t>
+  </si>
+  <si>
+    <t>Tiseyra</t>
+  </si>
+  <si>
+    <t>Isabella Giuliana</t>
+  </si>
+  <si>
+    <t>chidodejameempa@gmail.com</t>
+  </si>
+  <si>
+    <t>18/11/2010</t>
+  </si>
+  <si>
+    <t>Videla</t>
+  </si>
+  <si>
+    <t>Giuliana Abril</t>
+  </si>
+  <si>
+    <t>videlagiuliana4@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">Zapata </t>
   </si>
   <si>
-    <t xml:space="preserve">Ezequiel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ezequielzapatasantos@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docentes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">raularias@gmail.com</t>
+    <t>Ezequiel</t>
+  </si>
+  <si>
+    <t>ezequielzapatasantos@gmail.com</t>
+  </si>
+  <si>
+    <t>Docentes</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>Arias</t>
+  </si>
+  <si>
+    <t>Raul</t>
+  </si>
+  <si>
+    <t>raularias@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">Cantelli </t>
   </si>
   <si>
-    <t xml:space="preserve">Carolina Irene</t>
+    <t>Carolina Irene</t>
   </si>
   <si>
     <t xml:space="preserve">ccantelli@abc.gob.ar </t>
   </si>
   <si>
-    <t xml:space="preserve">Nelson Gabriel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gcasas1972@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gaston</t>
-  </si>
-  <si>
-    <t xml:space="preserve">profesorcuencagaston@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">da Costa Cardante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">David Alejandro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aleedacosta@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Damas Rendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juan Manuel</t>
+    <t>Nelson Gabriel</t>
+  </si>
+  <si>
+    <t>gcasas1972@gmail.com</t>
+  </si>
+  <si>
+    <t>Gaston</t>
+  </si>
+  <si>
+    <t>profesorcuencagaston@gmail.com</t>
+  </si>
+  <si>
+    <t>da Costa Cardante</t>
+  </si>
+  <si>
+    <t>David Alejandro</t>
+  </si>
+  <si>
+    <t>aleedacosta@gmail.com</t>
+  </si>
+  <si>
+    <t>Damas Rendon</t>
+  </si>
+  <si>
+    <t>Juan Manuel</t>
   </si>
   <si>
     <t xml:space="preserve"> noemirojas6666@gmail.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Julo Javier</t>
+    <t>Julo Javier</t>
   </si>
   <si>
     <t xml:space="preserve">jmolinero@abc.gob.ar </t>
   </si>
   <si>
-    <t xml:space="preserve">Maximiliano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pagesmaximiliano@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PARDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noemí</t>
+    <t>Maximiliano</t>
+  </si>
+  <si>
+    <t>pagesmaximiliano@gmail.com</t>
+  </si>
+  <si>
+    <t>PARDO</t>
+  </si>
+  <si>
+    <t>Noemí</t>
   </si>
   <si>
     <t xml:space="preserve">noemirojas6666@gmail.com </t>
@@ -527,130 +531,106 @@
     <t xml:space="preserve">Serrano </t>
   </si>
   <si>
-    <t xml:space="preserve">Serranofacundoignacio@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://plataforma.coparobotica.com/login?KJO-056</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pws</t>
+    <t>Serranofacundoignacio@gmail.com</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>https://plataforma.coparobotica.com/login?KJO-056</t>
+  </si>
+  <si>
+    <t>pws</t>
   </si>
   <si>
     <t xml:space="preserve">CUE </t>
   </si>
   <si>
-    <t xml:space="preserve">0690010/00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In4c-c14t4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">usu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avionica-ciata@faa.mil.ar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avionica-ciata@faa.mil.ar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pwd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">correo de la fuerza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://webcorreo.faa.mil.ar/</t>
+    <t>0690010/00</t>
+  </si>
+  <si>
+    <t>In4c-c14t4</t>
+  </si>
+  <si>
+    <t>usu</t>
+  </si>
+  <si>
+    <t>Avionica-ciata@faa.mil.ar</t>
+  </si>
+  <si>
+    <t>avionica-ciata@faa.mil.ar</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>pwd</t>
+  </si>
+  <si>
+    <t>correo de la fuerza</t>
+  </si>
+  <si>
+    <t>https://webcorreo.faa.mil.ar/</t>
   </si>
   <si>
     <t xml:space="preserve"> avionica-ciata@faa.mil.ar</t>
   </si>
   <si>
-    <t xml:space="preserve">bl20235512913</t>
-  </si>
-  <si>
-    <t xml:space="preserve">profesor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">telefonos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">edad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">joaquin.alcaraz.arosdecebolla@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carabajal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dylan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chucusea Quiroga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Correa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santino</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dacosta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Martinez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fabrizio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isabella giuliana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">presente</t>
+    <t>bl20235512913</t>
+  </si>
+  <si>
+    <t>Carabajal</t>
+  </si>
+  <si>
+    <t>Dylan</t>
+  </si>
+  <si>
+    <t>Chucusea Quiroga</t>
+  </si>
+  <si>
+    <t>Correa</t>
+  </si>
+  <si>
+    <t>Santino</t>
+  </si>
+  <si>
+    <t>Martinez</t>
+  </si>
+  <si>
+    <t>fabrizio</t>
+  </si>
+  <si>
+    <t>isabella giuliana</t>
+  </si>
+  <si>
+    <t>presente</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>muelte</t>
+  </si>
+  <si>
+    <t>se retiraron antes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
-    <numFmt numFmtId="166" formatCode="@"/>
-    <numFmt numFmtId="167" formatCode="dd\-mmm"/>
-    <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
+    <numFmt numFmtId="165" formatCode="dd\-mmm"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <u val="single"/>
+      <u/>
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
@@ -680,8 +660,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -736,9 +722,15 @@
         <bgColor rgb="FF993300"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -746,261 +738,101 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="57">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="54">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1059,62 +891,78 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1167,28 +1015,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:BY1048576"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:BY60"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="71.14"/>
+    <col min="1" max="1" width="4" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="1" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="32.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="71.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:77" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1196,7 +1043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1233,12 +1080,12 @@
       <c r="L2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="M2" s="2">
         <v>46142</v>
       </c>
     </row>
-    <row r="3" s="8" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="n">
+    <row r="3" spans="1:77" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
         <v>3</v>
       </c>
       <c r="B3" s="4" t="s">
@@ -1247,14 +1094,14 @@
       <c r="C3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="3">
         <v>50717603</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="6">
         <v>40505</v>
       </c>
       <c r="H3" s="4" t="s">
@@ -1340,38 +1187,38 @@
       <c r="BX3" s="7"/>
       <c r="BY3" s="7"/>
     </row>
-    <row r="4" s="13" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>50507317</v>
-      </c>
-      <c r="E4" s="8"/>
-      <c r="F4" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="10" t="n">
-        <v>40375</v>
-      </c>
-      <c r="H4" s="11" t="s">
+    <row r="4" spans="1:77" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>10</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" s="5">
+        <v>50658293</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>97</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="I4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>27</v>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="M4" s="7" t="s">
         <v>22</v>
@@ -1441,38 +1288,36 @@
       <c r="BX4" s="7"/>
       <c r="BY4" s="7"/>
     </row>
-    <row r="5" s="3" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="n">
-        <v>31</v>
-      </c>
-      <c r="B5" s="15" t="s">
+    <row r="5" spans="1:77" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
         <v>28</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="15" t="n">
-        <v>50981123</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="14" t="s">
+      <c r="B5" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" s="5">
+        <v>95622238</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="G5" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="L5" s="14" t="s">
-        <v>33</v>
+      <c r="K5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>22</v>
@@ -1542,39 +1387,38 @@
       <c r="BX5" s="7"/>
       <c r="BY5" s="7"/>
     </row>
-    <row r="6" s="14" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>50142917</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="14" t="s">
+    <row r="6" spans="1:77" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="3">
+        <v>50717565</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="33" t="s">
+        <v>106</v>
+      </c>
+      <c r="G6" s="6">
+        <v>40506</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="K6" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="L6" s="14" t="s">
-        <v>33</v>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>22</v>
@@ -1644,38 +1488,38 @@
       <c r="BX6" s="7"/>
       <c r="BY6" s="7"/>
     </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="18" t="n">
-        <v>49927919</v>
-      </c>
-      <c r="E7" s="18"/>
-      <c r="F7" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18" t="s">
+    <row r="7" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A7" s="34">
+        <v>29</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7" s="5">
+        <v>50353508</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G7" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="I7" s="18" t="s">
+      <c r="I7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="K7" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="L7" s="18" t="s">
-        <v>45</v>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>22</v>
@@ -1745,33 +1589,38 @@
       <c r="BX7" s="7"/>
       <c r="BY7" s="7"/>
     </row>
-    <row r="8" s="18" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="n">
+    <row r="8" spans="1:77" s="18" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>1</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="8">
+        <v>49810411</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="18" t="n">
-        <v>50987882</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="I8" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="K8" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="L8" s="18" t="s">
-        <v>45</v>
+      <c r="J8" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>27</v>
       </c>
       <c r="M8" s="7" t="s">
         <v>22</v>
@@ -1841,36 +1690,38 @@
       <c r="BX8" s="7"/>
       <c r="BY8" s="7"/>
     </row>
-    <row r="9" s="20" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>4973505</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="I9" s="20" t="s">
+    <row r="9" spans="1:77" s="20" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>9</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="8">
+        <v>50507317</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="10">
+        <v>40375</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="L9" s="20" t="s">
-        <v>55</v>
+      <c r="J9" s="8"/>
+      <c r="K9" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>27</v>
       </c>
       <c r="M9" s="7" t="s">
         <v>22</v>
@@ -1940,23 +1791,26 @@
       <c r="BX9" s="7"/>
       <c r="BY9" s="7"/>
     </row>
-    <row r="10" s="8" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
-        <v>22</v>
+    <row r="10" spans="1:77" s="8" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>15</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>57</v>
       </c>
+      <c r="D10" s="8">
+        <v>50686604</v>
+      </c>
       <c r="F10" s="9" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I10" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="8" t="s">
         <v>18</v>
       </c>
       <c r="K10" s="12" t="s">
@@ -2033,38 +1887,38 @@
       <c r="BX10" s="7"/>
       <c r="BY10" s="7"/>
     </row>
-    <row r="11" s="3" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="n">
-        <v>32</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" s="23" t="n">
-        <v>49521904</v>
-      </c>
-      <c r="E11" s="13"/>
-      <c r="F11" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="G11" s="24" t="n">
-        <v>40038</v>
-      </c>
-      <c r="H11" s="13" t="s">
+    <row r="11" spans="1:77" s="3" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>20</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" s="8">
+        <v>50276004</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="L11" s="13" t="s">
-        <v>63</v>
+      <c r="J11" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L11" s="11" t="s">
+        <v>27</v>
       </c>
       <c r="M11" s="7" t="s">
         <v>22</v>
@@ -2134,38 +1988,34 @@
       <c r="BX11" s="7"/>
       <c r="BY11" s="7"/>
     </row>
-    <row r="12" s="14" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="n">
-        <v>33</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12" s="23" t="n">
-        <v>48183416</v>
-      </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="G12" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H12" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="I12" s="13" t="s">
+    <row r="12" spans="1:77" s="14" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>22</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="L12" s="13" t="s">
-        <v>63</v>
+      <c r="J12" s="8"/>
+      <c r="K12" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>27</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>22</v>
@@ -2235,38 +2085,38 @@
       <c r="BX12" s="7"/>
       <c r="BY12" s="7"/>
     </row>
-    <row r="13" s="3" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="n">
-        <v>25</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" s="20" t="n">
-        <v>50141365</v>
-      </c>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="G13" s="26" t="n">
-        <v>40258</v>
-      </c>
-      <c r="H13" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="I13" s="20" t="s">
+    <row r="13" spans="1:77" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="13">
+        <v>2</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="13">
+        <v>49521627</v>
+      </c>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="28">
+        <v>39961</v>
+      </c>
+      <c r="H13" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="I13" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="20"/>
-      <c r="K13" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="L13" s="20" t="s">
-        <v>55</v>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L13" s="13" t="s">
+        <v>63</v>
       </c>
       <c r="M13" s="7" t="s">
         <v>22</v>
@@ -2336,38 +2186,38 @@
       <c r="BX13" s="7"/>
       <c r="BY13" s="7"/>
     </row>
-    <row r="14" s="14" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>49810411</v>
-      </c>
-      <c r="E14" s="8"/>
-      <c r="F14" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8" t="s">
+    <row r="14" spans="1:77" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="13">
+        <v>32</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="23">
+        <v>49521904</v>
+      </c>
+      <c r="E14" s="13"/>
+      <c r="F14" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="24">
+        <v>40038</v>
+      </c>
+      <c r="H14" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="K14" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>27</v>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L14" s="13" t="s">
+        <v>63</v>
       </c>
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
@@ -2435,30 +2285,30 @@
       <c r="BX14" s="7"/>
       <c r="BY14" s="7"/>
     </row>
-    <row r="15" s="14" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="n">
-        <v>2</v>
+    <row r="15" spans="1:77" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="13">
+        <v>23</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>49521627</v>
+        <v>130</v>
+      </c>
+      <c r="D15" s="13">
+        <v>49626775</v>
       </c>
       <c r="E15" s="13"/>
-      <c r="F15" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>39961</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="I15" s="13" t="s">
+      <c r="F15" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="G15" s="28">
+        <v>40065</v>
+      </c>
+      <c r="H15" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="I15" s="36" t="s">
         <v>18</v>
       </c>
       <c r="J15" s="13"/>
@@ -2534,40 +2384,38 @@
       <c r="BX15" s="7"/>
       <c r="BY15" s="7"/>
     </row>
-    <row r="16" s="8" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>50256549</v>
-      </c>
-      <c r="E16" s="14"/>
-      <c r="F16" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="G16" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="I16" s="14" t="s">
+    <row r="16" spans="1:77" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="13">
+        <v>24</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="D16" s="13">
+        <v>50490163</v>
+      </c>
+      <c r="E16" s="13"/>
+      <c r="F16" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="G16" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="K16" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>33</v>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L16" s="13" t="s">
+        <v>63</v>
       </c>
       <c r="M16" s="7"/>
       <c r="N16" s="7"/>
@@ -2635,38 +2483,38 @@
       <c r="BX16" s="7"/>
       <c r="BY16" s="7"/>
     </row>
-    <row r="17" s="18" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="D17" s="20" t="n">
-        <v>49001269</v>
-      </c>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="G17" s="26" t="n">
-        <v>39805</v>
-      </c>
-      <c r="H17" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="I17" s="20" t="s">
+    <row r="17" spans="1:77" s="18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="13">
+        <v>33</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="23">
+        <v>48183416</v>
+      </c>
+      <c r="E17" s="13"/>
+      <c r="F17" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="H17" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="I17" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="L17" s="20" t="s">
-        <v>55</v>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L17" s="13" t="s">
+        <v>63</v>
       </c>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
@@ -2734,8 +2582,8 @@
       <c r="BX17" s="7"/>
       <c r="BY17" s="7"/>
     </row>
-    <row r="18" s="18" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="n">
+    <row r="18" spans="1:77" s="18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="18">
         <v>7</v>
       </c>
       <c r="B18" s="18" t="s">
@@ -2744,7 +2592,7 @@
       <c r="C18" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="D18" s="18" t="n">
+      <c r="D18" s="18">
         <v>50276187</v>
       </c>
       <c r="F18" s="19" t="s">
@@ -2828,38 +2676,36 @@
       <c r="BX18" s="7"/>
       <c r="BY18" s="7"/>
     </row>
-    <row r="19" s="18" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="D19" s="20" t="n">
-        <v>49419297</v>
-      </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="G19" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="H19" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="I19" s="20" t="s">
+    <row r="19" spans="1:77" s="18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="18">
+        <v>16</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" s="18">
+        <v>49602531</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="I19" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="L19" s="20" t="s">
-        <v>55</v>
+      <c r="J19" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="K19" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="L19" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
@@ -2927,38 +2773,38 @@
       <c r="BX19" s="7"/>
       <c r="BY19" s="7"/>
     </row>
-    <row r="20" s="20" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>50658293</v>
-      </c>
-      <c r="E20" s="5"/>
-      <c r="F20" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="G20" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="H20" s="4" t="s">
+    <row r="20" spans="1:77" s="20" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="18">
         <v>17</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="B20" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="18">
+        <v>49927919</v>
+      </c>
+      <c r="E20" s="18"/>
+      <c r="F20" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="I20" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>21</v>
+      <c r="J20" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="L20" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
@@ -3026,38 +2872,36 @@
       <c r="BX20" s="7"/>
       <c r="BY20" s="7"/>
     </row>
-    <row r="21" s="8" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="B21" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="D21" s="14" t="n">
-        <v>49960662</v>
-      </c>
-      <c r="E21" s="14"/>
-      <c r="F21" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="G21" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="H21" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="I21" s="32" t="s">
+    <row r="21" spans="1:77" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="18">
         <v>18</v>
       </c>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="L21" s="14" t="s">
-        <v>33</v>
+      <c r="B21" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="18">
+        <v>50987882</v>
+      </c>
+      <c r="E21" s="18"/>
+      <c r="F21" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="L21" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="M21" s="7"/>
       <c r="N21" s="7"/>
@@ -3125,38 +2969,32 @@
       <c r="BX21" s="7"/>
       <c r="BY21" s="7"/>
     </row>
-    <row r="22" s="14" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>95622238</v>
-      </c>
-      <c r="E22" s="3"/>
-      <c r="F22" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="G22" s="31" t="s">
-        <v>103</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>21</v>
+    <row r="22" spans="1:77" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="18">
+        <v>27</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="L22" s="18" t="s">
+        <v>45</v>
       </c>
       <c r="M22" s="7"/>
       <c r="N22" s="7"/>
@@ -3224,38 +3062,38 @@
       <c r="BX22" s="7"/>
       <c r="BY22" s="7"/>
     </row>
-    <row r="23" s="8" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>50717565</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>40506</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I23" s="4" t="s">
+    <row r="23" spans="1:77" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="20">
+        <v>6</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="20">
+        <v>49001269</v>
+      </c>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="G23" s="26">
+        <v>39805</v>
+      </c>
+      <c r="H23" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="I23" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>21</v>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="L23" s="20" t="s">
+        <v>55</v>
       </c>
       <c r="M23" s="7"/>
       <c r="N23" s="7"/>
@@ -3323,38 +3161,38 @@
       <c r="BX23" s="7"/>
       <c r="BY23" s="7"/>
     </row>
-    <row r="24" s="13" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="n">
-        <v>14</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="D24" s="14" t="n">
-        <v>50656018</v>
-      </c>
-      <c r="E24" s="14"/>
-      <c r="F24" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="G24" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="I24" s="14" t="s">
+    <row r="24" spans="1:77" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="20">
+        <v>8</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D24" s="20">
+        <v>49419297</v>
+      </c>
+      <c r="E24" s="20"/>
+      <c r="F24" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="G24" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="H24" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="I24" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="L24" s="14" t="s">
-        <v>33</v>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="L24" s="20" t="s">
+        <v>55</v>
       </c>
       <c r="M24" s="7"/>
       <c r="N24" s="7"/>
@@ -3422,36 +3260,38 @@
       <c r="BX24" s="7"/>
       <c r="BY24" s="7"/>
     </row>
-    <row r="25" s="13" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D25" s="8" t="n">
-        <v>50686604</v>
-      </c>
-      <c r="E25" s="8"/>
-      <c r="F25" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I25" s="8" t="s">
+    <row r="25" spans="1:77" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="20">
+        <v>19</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="20">
+        <v>4973505</v>
+      </c>
+      <c r="E25" s="20"/>
+      <c r="F25" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="G25" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="H25" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="I25" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="J25" s="8"/>
-      <c r="K25" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="L25" s="11" t="s">
-        <v>27</v>
+      <c r="J25" s="20"/>
+      <c r="K25" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="L25" s="20" t="s">
+        <v>55</v>
       </c>
       <c r="M25" s="7"/>
       <c r="N25" s="7"/>
@@ -3519,38 +3359,36 @@
       <c r="BX25" s="7"/>
       <c r="BY25" s="7"/>
     </row>
-    <row r="26" s="20" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="n">
-        <v>16</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="D26" s="18" t="n">
-        <v>49602531</v>
-      </c>
-      <c r="E26" s="18"/>
-      <c r="F26" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="I26" s="18" t="s">
+    <row r="26" spans="1:77" s="20" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="20">
+        <v>25</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="20">
+        <v>50141365</v>
+      </c>
+      <c r="F26" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="G26" s="26">
+        <v>40258</v>
+      </c>
+      <c r="H26" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="I26" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="J26" s="18" t="s">
-        <v>116</v>
-      </c>
-      <c r="K26" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="L26" s="18" t="s">
-        <v>45</v>
+      <c r="K26" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="L26" s="20" t="s">
+        <v>55</v>
       </c>
       <c r="M26" s="7"/>
       <c r="N26" s="7"/>
@@ -3618,38 +3456,36 @@
       <c r="BX26" s="7"/>
       <c r="BY26" s="7"/>
     </row>
-    <row r="27" s="20" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D27" s="8" t="n">
-        <v>50276004</v>
-      </c>
-      <c r="E27" s="8"/>
-      <c r="F27" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8" t="s">
+    <row r="27" spans="1:77" s="20" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="20">
+        <v>26</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="D27" s="20">
+        <v>49676632</v>
+      </c>
+      <c r="F27" s="21" t="s">
+        <v>138</v>
+      </c>
+      <c r="G27" s="37">
+        <v>40032</v>
+      </c>
+      <c r="H27" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="I27" s="8" t="s">
+      <c r="I27" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="J27" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="K27" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="L27" s="11" t="s">
-        <v>27</v>
+      <c r="K27" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="L27" s="38" t="s">
+        <v>55</v>
       </c>
       <c r="M27" s="7"/>
       <c r="N27" s="7"/>
@@ -3717,25 +3553,25 @@
       <c r="BX27" s="7"/>
       <c r="BY27" s="7"/>
     </row>
-    <row r="28" s="18" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="n">
-        <v>21</v>
+    <row r="28" spans="1:77" s="18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="14">
+        <v>4</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="D28" s="14" t="n">
-        <v>49804684</v>
+        <v>80</v>
+      </c>
+      <c r="D28" s="14">
+        <v>50256549</v>
       </c>
       <c r="E28" s="14"/>
-      <c r="F28" s="15" t="s">
-        <v>123</v>
+      <c r="F28" s="29" t="s">
+        <v>81</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="H28" s="14" t="s">
         <v>38</v>
@@ -3743,7 +3579,9 @@
       <c r="I28" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="J28" s="14"/>
+      <c r="J28" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="K28" s="14" t="s">
         <v>32</v>
       </c>
@@ -3816,36 +3654,38 @@
       <c r="BX28" s="7"/>
       <c r="BY28" s="7"/>
     </row>
-    <row r="29" s="3" customFormat="true" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="34" t="n">
-        <v>29</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>50353508</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="G29" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="H29" s="3" t="s">
+    <row r="29" spans="1:77" s="3" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="14">
+        <v>11</v>
+      </c>
+      <c r="B29" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D29" s="14">
+        <v>49960662</v>
+      </c>
+      <c r="E29" s="14"/>
+      <c r="F29" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H29" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="I29" s="3" t="s">
+      <c r="I29" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="K29" s="3" t="s">
+      <c r="J29" s="14"/>
+      <c r="K29" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="L29" s="3" t="s">
-        <v>21</v>
+      <c r="L29" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="M29" s="7"/>
       <c r="N29" s="7"/>
@@ -3913,38 +3753,38 @@
       <c r="BX29" s="7"/>
       <c r="BY29" s="7"/>
     </row>
-    <row r="30" s="3" customFormat="true" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="n">
-        <v>23</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="D30" s="13" t="n">
-        <v>49626775</v>
-      </c>
-      <c r="E30" s="13"/>
-      <c r="F30" s="35" t="s">
-        <v>131</v>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>40065</v>
-      </c>
-      <c r="H30" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="I30" s="36" t="s">
+    <row r="30" spans="1:77" s="3" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="14">
+        <v>31</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" s="15">
+        <v>50981123</v>
+      </c>
+      <c r="E30" s="14"/>
+      <c r="F30" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="G30" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H30" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="J30" s="13"/>
-      <c r="K30" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="L30" s="13" t="s">
-        <v>63</v>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="L30" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="M30" s="7"/>
       <c r="N30" s="7"/>
@@ -4012,38 +3852,39 @@
       <c r="BX30" s="7"/>
       <c r="BY30" s="7"/>
     </row>
-    <row r="31" s="14" customFormat="true" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="n">
-        <v>24</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="D31" s="13" t="n">
-        <v>50490163</v>
-      </c>
-      <c r="E31" s="13"/>
-      <c r="F31" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="G31" s="25" t="s">
-        <v>135</v>
-      </c>
-      <c r="H31" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="I31" s="13" t="s">
+    <row r="31" spans="1:77" s="14" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="14">
+        <v>13</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" s="14">
+        <v>50142917</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="I31" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="J31" s="13"/>
-      <c r="K31" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="L31" s="13" t="s">
-        <v>63</v>
+      <c r="J31" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="K31" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="L31" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="M31" s="7"/>
       <c r="N31" s="7"/>
@@ -4111,38 +3952,38 @@
       <c r="BX31" s="7"/>
       <c r="BY31" s="7"/>
     </row>
-    <row r="32" s="13" customFormat="true" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="n">
-        <v>26</v>
-      </c>
-      <c r="B32" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="D32" s="20" t="n">
-        <v>49676632</v>
-      </c>
-      <c r="E32" s="20"/>
-      <c r="F32" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="G32" s="37" t="n">
-        <v>40032</v>
-      </c>
-      <c r="H32" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="I32" s="20" t="s">
+    <row r="32" spans="1:77" s="13" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="14">
+        <v>14</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="D32" s="14">
+        <v>50656018</v>
+      </c>
+      <c r="E32" s="14"/>
+      <c r="F32" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="G32" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="J32" s="20"/>
-      <c r="K32" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="L32" s="38" t="s">
-        <v>55</v>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="L32" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="M32" s="7"/>
       <c r="N32" s="7"/>
@@ -4210,32 +4051,38 @@
       <c r="BX32" s="7"/>
       <c r="BY32" s="7"/>
     </row>
-    <row r="33" s="13" customFormat="true" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="C33" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="I33" s="18"/>
-      <c r="J33" s="18"/>
-      <c r="K33" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="L33" s="18" t="s">
-        <v>45</v>
+    <row r="33" spans="1:77" s="13" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="14">
+        <v>21</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="D33" s="14">
+        <v>49804684</v>
+      </c>
+      <c r="E33" s="14"/>
+      <c r="F33" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="G33" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="H33" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="L33" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="M33" s="7"/>
       <c r="N33" s="7"/>
@@ -4303,23 +4150,23 @@
       <c r="BX33" s="7"/>
       <c r="BY33" s="7"/>
     </row>
-    <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:77" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="39"/>
       <c r="C34" s="39"/>
       <c r="D34" s="39"/>
       <c r="F34" s="39"/>
       <c r="G34" s="40"/>
-      <c r="M34" s="1" t="n">
-        <f aca="false">COUNTIF(M3:M33,"P")</f>
+      <c r="M34" s="1">
+        <f>COUNTIF(M3:M33,"P")</f>
         <v>11</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:77" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:77" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
         <v>3</v>
       </c>
@@ -4336,8 +4183,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="n">
+    <row r="39" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
         <v>1</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -4346,18 +4193,18 @@
       <c r="C39" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D39" s="1" t="n">
+      <c r="D39" s="1">
         <v>21491938</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="G39" s="2" t="n">
+      <c r="G39" s="2">
         <v>25749</v>
       </c>
     </row>
-    <row r="40" s="3" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="n">
+    <row r="40" spans="1:77" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
         <v>2</v>
       </c>
       <c r="B40" s="3" t="s">
@@ -4366,20 +4213,20 @@
       <c r="C40" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="D40" s="3" t="n">
+      <c r="D40" s="3">
         <v>23887042</v>
       </c>
       <c r="F40" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="G40" s="6" t="n">
+      <c r="G40" s="6">
         <v>27085</v>
       </c>
       <c r="Q40" s="1"/>
       <c r="R40" s="1"/>
     </row>
-    <row r="41" s="8" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="8" t="n">
+    <row r="41" spans="1:77" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="8">
         <v>3</v>
       </c>
       <c r="B41" s="8" t="s">
@@ -4388,20 +4235,20 @@
       <c r="C41" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="D41" s="8" t="n">
+      <c r="D41" s="8">
         <v>22965726</v>
       </c>
       <c r="F41" s="27" t="s">
         <v>151</v>
       </c>
-      <c r="G41" s="10" t="n">
+      <c r="G41" s="10">
         <v>26620</v>
       </c>
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
     </row>
-    <row r="42" s="41" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="41" t="n">
+    <row r="42" spans="1:77" s="41" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="41">
         <v>4</v>
       </c>
       <c r="B42" s="42" t="s">
@@ -4410,20 +4257,20 @@
       <c r="C42" s="41" t="s">
         <v>152</v>
       </c>
-      <c r="D42" s="41" t="n">
+      <c r="D42" s="41">
         <v>34576597</v>
       </c>
       <c r="F42" s="43" t="s">
         <v>153</v>
       </c>
-      <c r="G42" s="44" t="n">
+      <c r="G42" s="44">
         <v>32683</v>
       </c>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
     </row>
-    <row r="43" s="18" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="18" t="n">
+    <row r="43" spans="1:77" s="18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="18">
         <v>5</v>
       </c>
       <c r="B43" s="18" t="s">
@@ -4432,20 +4279,20 @@
       <c r="C43" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="D43" s="18" t="n">
+      <c r="D43" s="18">
         <v>40090104</v>
       </c>
       <c r="F43" s="45" t="s">
         <v>156</v>
       </c>
-      <c r="G43" s="46" t="n">
+      <c r="G43" s="46">
         <v>35478</v>
       </c>
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
     </row>
-    <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1" t="n">
+    <row r="44" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
         <v>6</v>
       </c>
       <c r="B44" s="1" t="s">
@@ -4454,18 +4301,18 @@
       <c r="C44" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D44" s="1" t="n">
+      <c r="D44" s="1">
         <v>45465583</v>
       </c>
       <c r="F44" s="47" t="s">
         <v>159</v>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="G44" s="2">
         <v>29268</v>
       </c>
     </row>
-    <row r="45" s="20" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="20" t="n">
+    <row r="45" spans="1:77" s="20" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="20">
         <v>7</v>
       </c>
       <c r="B45" s="20" t="s">
@@ -4474,20 +4321,20 @@
       <c r="C45" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="D45" s="20" t="n">
+      <c r="D45" s="20">
         <v>26971538</v>
       </c>
       <c r="F45" s="48" t="s">
         <v>161</v>
       </c>
-      <c r="G45" s="26" t="n">
+      <c r="G45" s="26">
         <v>28784</v>
       </c>
       <c r="Q45" s="1"/>
       <c r="R45" s="1"/>
     </row>
-    <row r="46" s="14" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="14" t="n">
+    <row r="46" spans="1:77" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="14">
         <v>8</v>
       </c>
       <c r="B46" s="14" t="s">
@@ -4496,20 +4343,20 @@
       <c r="C46" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="D46" s="14" t="n">
+      <c r="D46" s="14">
         <v>36735810</v>
       </c>
       <c r="F46" s="49" t="s">
         <v>163</v>
       </c>
-      <c r="G46" s="50" t="n">
+      <c r="G46" s="50">
         <v>33635</v>
       </c>
       <c r="Q46" s="1"/>
       <c r="R46" s="1"/>
     </row>
-    <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="1" t="n">
+    <row r="47" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
         <v>9</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -4518,18 +4365,18 @@
       <c r="C47" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D47" s="1" t="n">
+      <c r="D47" s="1">
         <v>27925268</v>
       </c>
       <c r="F47" s="47" t="s">
         <v>166</v>
       </c>
-      <c r="G47" s="2" t="n">
+      <c r="G47" s="2">
         <v>29268</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="1" t="n">
+    <row r="48" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
         <v>10</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -4538,29 +4385,29 @@
       <c r="C48" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D48" s="1" t="n">
+      <c r="D48" s="1">
         <v>41835642</v>
       </c>
       <c r="F48" s="47" t="s">
         <v>168</v>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="G48" s="2">
         <v>36262</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G49" s="2"/>
     </row>
-    <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="55" t="s">
         <v>170</v>
       </c>
       <c r="G50" s="2"/>
     </row>
-    <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>171</v>
       </c>
@@ -4574,11 +4421,11 @@
         <v>174</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="55" t="s">
         <v>176</v>
       </c>
       <c r="C52" s="1" t="s">
@@ -4588,7 +4435,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>175</v>
       </c>
@@ -4596,7 +4443,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>179</v>
       </c>
@@ -4604,12 +4451,12 @@
         <v>174</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>169</v>
       </c>
@@ -4617,7 +4464,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>175</v>
       </c>
@@ -4625,7 +4472,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>179</v>
       </c>
@@ -4633,32 +4480,34 @@
         <v>183</v>
       </c>
     </row>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
+  <sortState ref="A3:L33">
+    <sortCondition ref="L3:L33"/>
+    <sortCondition ref="B3:B33"/>
+  </sortState>
   <hyperlinks>
-    <hyperlink ref="F4" r:id="rId1" display="quiroruth1@gmail.com"/>
-    <hyperlink ref="F5" r:id="rId2" display="palofariasruiz@gmail.com"/>
-    <hyperlink ref="F7" r:id="rId3" display="thiaguitolujan09@gmail.com"/>
-    <hyperlink ref="F8" r:id="rId4" display="benicio.luna11@gmail.com"/>
-    <hyperlink ref="F10" r:id="rId5" display="mateoprado2701@gmail.com"/>
-    <hyperlink ref="F14" r:id="rId6" display="Ven09130814@gmail.com"/>
-    <hyperlink ref="F16" r:id="rId7" display="arredondofacundo406@gmail.com"/>
-    <hyperlink ref="F18" r:id="rId8" display="ulimirage3@gmail.com"/>
-    <hyperlink ref="F23" r:id="rId9" display="punaxs31@gmail.com"/>
-    <hyperlink ref="F25" r:id="rId10" display="mateobautistalescano123@gmail.com"/>
-    <hyperlink ref="F26" r:id="rId11" display="valentinluceroxd@gmail.com"/>
-    <hyperlink ref="F27" r:id="rId12" display="tahiel.e.manrique@gmail.com"/>
-    <hyperlink ref="F30" r:id="rId13" display="ven09130814@gmail.com"/>
-    <hyperlink ref="F33" r:id="rId14" display="ezequielzapatasantos@gmail.com"/>
-    <hyperlink ref="F41" r:id="rId15" display="gcasas1972@gmail.com"/>
-    <hyperlink ref="B54" r:id="rId16" display="gcasas1972@gmail.com"/>
+    <hyperlink ref="F9" r:id="rId1"/>
+    <hyperlink ref="F30" r:id="rId2"/>
+    <hyperlink ref="F20" r:id="rId3"/>
+    <hyperlink ref="F21" r:id="rId4"/>
+    <hyperlink ref="F12" r:id="rId5"/>
+    <hyperlink ref="F8" r:id="rId6"/>
+    <hyperlink ref="F28" r:id="rId7"/>
+    <hyperlink ref="F18" r:id="rId8"/>
+    <hyperlink ref="F6" r:id="rId9"/>
+    <hyperlink ref="F10" r:id="rId10"/>
+    <hyperlink ref="F19" r:id="rId11"/>
+    <hyperlink ref="F11" r:id="rId12"/>
+    <hyperlink ref="F15" r:id="rId13"/>
+    <hyperlink ref="F22" r:id="rId14"/>
+    <hyperlink ref="F41" r:id="rId15"/>
+    <hyperlink ref="B54" r:id="rId16"/>
+    <hyperlink ref="B50" r:id="rId17"/>
+    <hyperlink ref="B52" r:id="rId18"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>
@@ -4666,21 +4515,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:K29"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="36.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="33.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12.29"/>
+    <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4693,30 +4538,18 @@
       <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>143</v>
+      <c r="E1" s="51">
+        <v>46135</v>
+      </c>
+      <c r="F1" s="52">
+        <v>46149</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="K1" s="51" t="n">
-        <v>46135</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -4728,18 +4561,15 @@
       <c r="D2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="52" t="s">
-        <v>187</v>
-      </c>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="52"/>
-      <c r="K2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
+      <c r="F2" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -4751,9 +4581,12 @@
       <c r="D3" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+      <c r="F3" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -4765,9 +4598,12 @@
       <c r="D4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
+      <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -4779,35 +4615,36 @@
       <c r="D5" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="52" t="s">
-        <v>81</v>
-      </c>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
+      <c r="F5" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="53">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="B6" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" s="53" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="n">
+      <c r="E6" s="53"/>
+      <c r="F6" s="53" t="s">
+        <v>193</v>
+      </c>
+      <c r="G6" s="54" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -4819,9 +4656,12 @@
       <c r="D7" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
+      <c r="F7" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -4833,28 +4673,15 @@
       <c r="D8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="1" t="n">
-        <v>50276187</v>
-      </c>
-      <c r="F8" s="52" t="s">
-        <v>89</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="53" t="n">
-        <v>40324</v>
-      </c>
-      <c r="I8" s="52"/>
-      <c r="J8" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
+      <c r="F8" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -4866,13 +4693,16 @@
       <c r="D9" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="n">
+      <c r="F9" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>24</v>
@@ -4880,32 +4710,35 @@
       <c r="D10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="52" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="52"/>
-      <c r="H10" s="52"/>
-      <c r="I10" s="52"/>
-      <c r="K10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="n">
+      <c r="F10" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="n">
+      <c r="F11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -4917,9 +4750,13 @@
       <c r="D12" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="n">
+      <c r="F12" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="G12" s="56"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -4931,21 +4768,15 @@
       <c r="D13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="52" t="s">
-        <v>106</v>
-      </c>
-      <c r="G13" s="52"/>
-      <c r="H13" s="52"/>
-      <c r="I13" s="52"/>
-      <c r="J13" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K13" s="7" t="s">
+      <c r="E13" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="n">
+      <c r="F13" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -4957,9 +4788,12 @@
       <c r="D14" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="n">
+      <c r="F14" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -4971,9 +4805,12 @@
       <c r="D15" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="n">
+      <c r="F15" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -4985,21 +4822,18 @@
       <c r="D16" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="52" t="s">
-        <v>112</v>
-      </c>
-      <c r="G16" s="52"/>
-      <c r="H16" s="52"/>
-      <c r="I16" s="52"/>
-      <c r="J16" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="n">
+      <c r="F16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -5011,26 +4845,15 @@
       <c r="D17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="1" t="n">
-        <v>49602531</v>
-      </c>
-      <c r="F17" s="52" t="s">
-        <v>115</v>
-      </c>
-      <c r="G17" s="52"/>
-      <c r="H17" s="53" t="n">
-        <v>39931</v>
-      </c>
-      <c r="I17" s="52"/>
-      <c r="J17" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="K17" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+      <c r="F17" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -5042,28 +4865,15 @@
       <c r="D18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="1" t="n">
-        <v>49927919</v>
-      </c>
-      <c r="F18" s="52" t="s">
-        <v>42</v>
-      </c>
-      <c r="G18" s="7" t="s">
+      <c r="E18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H18" s="53" t="n">
-        <v>40165</v>
-      </c>
-      <c r="I18" s="52"/>
-      <c r="J18" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="n">
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -5075,21 +4885,15 @@
       <c r="D19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="52" t="s">
-        <v>48</v>
-      </c>
-      <c r="G19" s="52"/>
-      <c r="H19" s="52"/>
-      <c r="I19" s="52"/>
-      <c r="J19" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K19" s="7" t="s">
+      <c r="E19" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="n">
+      <c r="F19" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -5101,9 +4905,12 @@
       <c r="D20" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="n">
+      <c r="F20" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -5115,35 +4922,32 @@
       <c r="D21" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F21" s="52" t="s">
-        <v>119</v>
-      </c>
-      <c r="G21" s="52"/>
-      <c r="H21" s="52"/>
-      <c r="I21" s="52"/>
-      <c r="J21" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K21" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="n">
+      <c r="F21" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="n">
+      <c r="F22" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -5155,21 +4959,15 @@
       <c r="D23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F23" s="52" t="s">
-        <v>58</v>
-      </c>
-      <c r="G23" s="52"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="52"/>
-      <c r="J23" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="K23" s="7" t="s">
+      <c r="E23" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="n">
+      <c r="F23" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -5181,23 +4979,29 @@
       <c r="D24" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="n">
+      <c r="F24" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>132</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="n">
+      <c r="F25" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -5209,9 +5013,12 @@
       <c r="D26" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="n">
+      <c r="F26" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -5223,9 +5030,12 @@
       <c r="D27" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="n">
+      <c r="F27" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -5237,46 +5047,37 @@
       <c r="D28" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F28" s="52" t="s">
-        <v>141</v>
-      </c>
-      <c r="G28" s="52"/>
-      <c r="H28" s="52"/>
-      <c r="I28" s="52"/>
-      <c r="J28" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K28" s="7" t="s">
+      <c r="E28" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F28" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D29" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="K29" s="1" t="n">
-        <f aca="false">COUNTIF(K2:K28,"P")</f>
+        <v>192</v>
+      </c>
+      <c r="E29" s="1">
+        <f>COUNTIF(E2:E28,"P")</f>
         <v>12</v>
       </c>
+      <c r="F29" s="1">
+        <f>COUNTIF(F2:F28,"P")</f>
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F5" r:id="rId1" display="arredondofacundo406@gmail.com"/>
-    <hyperlink ref="F8" r:id="rId2" display="ulimirage3@gmail.com"/>
-    <hyperlink ref="F10" r:id="rId3" display="quiroruth1@gmail.com"/>
-    <hyperlink ref="F13" r:id="rId4" display="punaxs31@gmail.com"/>
-    <hyperlink ref="F16" r:id="rId5" display="mateobautistalescano123@gmail.com"/>
-    <hyperlink ref="F17" r:id="rId6" display="valentinluceroxd@gmail.com"/>
-    <hyperlink ref="F18" r:id="rId7" display="thiaguitolujan09@gmail.com"/>
-    <hyperlink ref="F19" r:id="rId8" display="benicio.luna11@gmail.com"/>
-    <hyperlink ref="F21" r:id="rId9" display="tahiel.e.manrique@gmail.com"/>
-    <hyperlink ref="F23" r:id="rId10" display="mateoprado2701@gmail.com"/>
-    <hyperlink ref="F28" r:id="rId11" display="ezequielzapatasantos@gmail.com"/>
-  </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <sortState ref="A2:G28">
+    <sortCondition ref="B2:B28"/>
+    <sortCondition ref="C2:C28"/>
+  </sortState>
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
agregado de minuta de reunion y actualizacion de asistencia
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="196">
   <si>
     <t>Alumnos</t>
   </si>
@@ -742,7 +742,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
@@ -826,6 +826,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -4516,7 +4517,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
@@ -4525,7 +4526,7 @@
     <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4547,8 +4548,11 @@
       <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" s="52">
+        <v>46156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -4567,8 +4571,11 @@
       <c r="F2" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -4584,8 +4591,11 @@
       <c r="F3" s="1" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -4601,8 +4611,11 @@
       <c r="F4" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -4621,8 +4634,11 @@
       <c r="F5" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="H5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="53">
         <v>5</v>
       </c>
@@ -4643,7 +4659,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -4659,8 +4675,11 @@
       <c r="F7" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -4679,8 +4698,11 @@
       <c r="F8" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -4696,8 +4718,11 @@
       <c r="F9" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -4716,8 +4741,11 @@
       <c r="F10" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -4736,8 +4764,11 @@
       <c r="G11" s="7" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H11" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -4754,8 +4785,11 @@
         <v>193</v>
       </c>
       <c r="G12" s="56"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H12" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -4774,8 +4808,11 @@
       <c r="F13" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H13" s="57" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -4791,8 +4828,11 @@
       <c r="F14" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H14" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -4808,8 +4848,11 @@
       <c r="F15" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H15" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -4831,8 +4874,11 @@
       <c r="G16" s="7" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H16" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -4842,17 +4888,20 @@
       <c r="C17" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="57" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H17" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -4862,17 +4911,20 @@
       <c r="C18" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="57" t="s">
         <v>22</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H18" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -4891,8 +4943,11 @@
       <c r="F19" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H19" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -4908,8 +4963,11 @@
       <c r="F20" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H20" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -4928,8 +4986,11 @@
       <c r="F21" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H21" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -4945,8 +5006,11 @@
       <c r="F22" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H22" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -4965,8 +5029,11 @@
       <c r="F23" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H23" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -4982,8 +5049,11 @@
       <c r="F24" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H24" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -4999,8 +5069,11 @@
       <c r="F25" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H25" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -5016,8 +5089,11 @@
       <c r="F26" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H26" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -5033,8 +5109,11 @@
       <c r="F27" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H27" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -5056,8 +5135,11 @@
       <c r="G28" s="7" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H28" s="7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="D29" s="1" t="s">
         <v>192</v>
       </c>
@@ -5069,9 +5151,13 @@
         <f>COUNTIF(F2:F28,"P")</f>
         <v>10</v>
       </c>
+      <c r="H29" s="1">
+        <f>COUNTIF(H2:H28,"P")</f>
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:G28">
+  <sortState ref="A2:H28">
     <sortCondition ref="B2:B28"/>
     <sortCondition ref="C2:C28"/>
   </sortState>

</xml_diff>

<commit_message>
agregado de minuta de reunion
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="200">
   <si>
     <t>Alumnos</t>
   </si>
@@ -613,6 +613,18 @@
   </si>
   <si>
     <t>se retiraron antes</t>
+  </si>
+  <si>
+    <t>prsentes</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>nota</t>
   </si>
 </sst>
 </file>
@@ -4517,16 +4529,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
     <col min="5" max="5" width="12.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
+    <col min="8" max="10" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4551,19 +4566,34 @@
       <c r="H1" s="52">
         <v>46156</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" s="52">
+        <v>46163</v>
+      </c>
+      <c r="J1" t="s">
+        <v>196</v>
+      </c>
+      <c r="K1" t="s">
+        <v>199</v>
+      </c>
+      <c r="L1">
+        <v>3</v>
+      </c>
+      <c r="M1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>71</v>
+        <v>186</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>22</v>
@@ -4572,61 +4602,109 @@
         <v>22</v>
       </c>
       <c r="H2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2">
+        <f>COUNTIF(E2:I2,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <f>ROUND(J2*10/4,0)</f>
+        <v>10</v>
+      </c>
+      <c r="L2" t="s">
+        <v>197</v>
+      </c>
+      <c r="M2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>75</v>
+        <v>111</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="H3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3">
+        <f>COUNTIF(E3:I3,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <f>ROUND(J3*10/4,0)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="E4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H4" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4">
+        <f>COUNTIF(E4:I4,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K4">
+        <f>ROUND(J4*10/4,0)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>22</v>
@@ -4635,62 +4713,101 @@
         <v>22</v>
       </c>
       <c r="H5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="53">
-        <v>5</v>
-      </c>
-      <c r="B6" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="C6" s="53" t="s">
-        <v>185</v>
-      </c>
-      <c r="D6" s="53" t="s">
+      <c r="J5">
+        <f>COUNTIF(E5:I5,"P")</f>
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <f>ROUND(J5*10/4,0)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53" t="s">
-        <v>193</v>
-      </c>
-      <c r="G6" s="54" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E6" s="1"/>
+      <c r="F6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6">
+        <f>COUNTIF(E6:I6,"P")</f>
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <f>ROUND(J6*10/4,0)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>78</v>
+        <v>17</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H7" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H7" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7">
+        <f>COUNTIF(E7:I7,"P")</f>
+        <v>3</v>
+      </c>
+      <c r="K7">
+        <f>ROUND(J7*10/4,0)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>22</v>
@@ -4699,41 +4816,63 @@
         <v>22</v>
       </c>
       <c r="H8" t="s">
+        <v>193</v>
+      </c>
+      <c r="I8" t="s">
+        <v>193</v>
+      </c>
+      <c r="J8">
+        <f>COUNTIF(E8:I8,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K8">
+        <f>ROUND(J8*10/4,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>193</v>
       </c>
       <c r="H9" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I9" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9">
+        <f>COUNTIF(E9:I9,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K9">
+        <f>ROUND(J9*10/4,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>186</v>
+        <v>79</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>22</v>
@@ -4742,18 +4881,29 @@
         <v>22</v>
       </c>
       <c r="H10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="I10" t="s">
+        <v>193</v>
+      </c>
+      <c r="J10">
+        <f>COUNTIF(E10:I10,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K10">
+        <f>ROUND(J10*10/4,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>187</v>
+        <v>132</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>17</v>
@@ -4761,69 +4911,105 @@
       <c r="F11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="7" t="s">
-        <v>195</v>
-      </c>
       <c r="H11" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I11" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J11">
+        <f>COUNTIF(E11:I11,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K11">
+        <f>ROUND(J11*10/4,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
+        <v>27</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J12">
+        <f>COUNTIF(E12:I12,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K12">
+        <f>ROUND(J12*10/4,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="G12" s="56"/>
-      <c r="H12" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>12</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>22</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H13" s="57" t="s">
+      <c r="G13" s="56"/>
+      <c r="H13" s="7" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I13" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J13">
+        <f>COUNTIF(E13:I13,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <f>ROUND(J13*10/4,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>34</v>
+        <v>113</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D14" s="57" t="s">
         <v>38</v>
+      </c>
+      <c r="E14" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>193</v>
@@ -4831,19 +5017,33 @@
       <c r="H14" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I14" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J14">
+        <f>COUNTIF(E14:I14,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <f>ROUND(J14*10/4,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>107</v>
+        <v>40</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
+      </c>
+      <c r="D15" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>193</v>
@@ -4851,47 +5051,66 @@
       <c r="H15" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I15" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J15">
+        <f>COUNTIF(E15:I15,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <f>ROUND(J15*10/4,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>57</v>
+        <v>118</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F16" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J16">
+        <f>COUNTIF(E16:I16,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <f>ROUND(J16*10/4,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>22</v>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>16</v>
-      </c>
       <c r="B17" s="1" t="s">
-        <v>113</v>
+        <v>56</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D17" s="57" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="57" t="s">
+      <c r="E17" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="7" t="s">
@@ -4900,151 +5119,216 @@
       <c r="H17" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I17" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J17">
+        <f>COUNTIF(E17:I17,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <f>ROUND(J17*10/4,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D18" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E18" s="57" t="s">
-        <v>22</v>
+        <v>69</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>193</v>
       </c>
       <c r="H18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="J18">
+        <f>COUNTIF(E18:I18,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <f>ROUND(J18*10/4,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="H19" t="s">
+        <v>193</v>
+      </c>
+      <c r="I19" t="s">
+        <v>193</v>
+      </c>
+      <c r="J19">
+        <f>COUNTIF(E19:I19,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <f>ROUND(J19*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="53">
+        <v>5</v>
+      </c>
+      <c r="B20" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="C20" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D20" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>19</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F20" s="7" t="s">
+      <c r="E20" s="53"/>
+      <c r="F20" s="53" t="s">
         <v>193</v>
       </c>
-      <c r="H20" s="7" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G20" s="54" t="s">
+        <v>194</v>
+      </c>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54"/>
+      <c r="J20">
+        <f>COUNTIF(E20:I20,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <f>ROUND(J20*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>117</v>
+        <v>84</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>118</v>
+        <v>85</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="H21" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I21" t="s">
+        <v>193</v>
+      </c>
+      <c r="J21">
+        <f>COUNTIF(E21:I21,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <f>ROUND(J21*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>189</v>
+        <v>90</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>190</v>
+        <v>91</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I22" t="s">
+        <v>193</v>
+      </c>
+      <c r="J22">
+        <f>COUNTIF(E22:I22,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <f>ROUND(J22*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E23" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F23" s="7" t="s">
         <v>193</v>
       </c>
       <c r="H23" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I23" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J23">
+        <f>COUNTIF(E23:I23,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <f>ROUND(J23*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>193</v>
@@ -5052,59 +5336,92 @@
       <c r="H24" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I24" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J24">
+        <f>COUNTIF(E24:I24,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <f>ROUND(J24*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>132</v>
+        <v>49</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>191</v>
+        <v>50</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J25">
+        <f>COUNTIF(E25:I25,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <f>ROUND(J25*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>64</v>
+        <v>189</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>69</v>
+        <v>190</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>193</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J26">
+        <f>COUNTIF(E26:I26,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <f>ROUND(J26*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>193</v>
@@ -5112,34 +5429,50 @@
       <c r="H27" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I27" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J27">
+        <f>COUNTIF(E27:I27,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <f>ROUND(J27*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I28" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J28">
+        <f>COUNTIF(E28:I28,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <f>ROUND(J28*10/4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D29" s="1" t="s">
         <v>192</v>
       </c>
@@ -5155,11 +5488,15 @@
         <f>COUNTIF(H2:H28,"P")</f>
         <v>9</v>
       </c>
+      <c r="I29" s="57">
+        <f>COUNTIF(I2:I28,"P")</f>
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:H28">
+  <sortState ref="A2:K28">
+    <sortCondition descending="1" ref="K2:K28"/>
     <sortCondition ref="B2:B28"/>
-    <sortCondition ref="C2:C28"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
agregado de documentacion y minuta de reunion
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="alumnos" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="204">
   <si>
     <t>Alumnos</t>
   </si>
@@ -618,13 +618,25 @@
     <t>prsentes</t>
   </si>
   <si>
-    <t>n</t>
-  </si>
-  <si>
     <t>x</t>
   </si>
   <si>
     <t>nota</t>
+  </si>
+  <si>
+    <t>Bustos Lisboa</t>
+  </si>
+  <si>
+    <t>2C</t>
+  </si>
+  <si>
+    <t>Salvador</t>
+  </si>
+  <si>
+    <t>Barzo Marchi</t>
+  </si>
+  <si>
+    <t>Juan</t>
   </si>
 </sst>
 </file>
@@ -4529,7 +4541,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
@@ -4573,10 +4585,10 @@
         <v>196</v>
       </c>
       <c r="K1" t="s">
-        <v>199</v>
-      </c>
-      <c r="L1">
-        <v>3</v>
+        <v>198</v>
+      </c>
+      <c r="L1" s="52">
+        <v>46177</v>
       </c>
       <c r="M1">
         <v>10</v>
@@ -4584,16 +4596,16 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>186</v>
+        <v>71</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>22</v>
@@ -4602,75 +4614,72 @@
         <v>22</v>
       </c>
       <c r="H2" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I2" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="J2">
         <f>COUNTIF(E2:I2,"P")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <f>ROUND(J2*10/4,0)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L2" t="s">
+        <v>193</v>
+      </c>
+      <c r="M2" t="s">
         <v>197</v>
-      </c>
-      <c r="M2" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>111</v>
+        <v>75</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>22</v>
+        <v>78</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="H3" t="s">
+        <v>193</v>
+      </c>
+      <c r="I3" t="s">
+        <v>193</v>
       </c>
       <c r="J3">
         <f>COUNTIF(E3:I3,"P")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K3">
         <f>ROUND(J3*10/4,0)</f>
-        <v>10</v>
+        <v>0</v>
+      </c>
+      <c r="L3" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>22</v>
@@ -4678,114 +4687,118 @@
       <c r="F4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>22</v>
+      <c r="H4" t="s">
+        <v>193</v>
+      </c>
+      <c r="I4" t="s">
+        <v>193</v>
       </c>
       <c r="J4">
         <f>COUNTIF(E4:I4,"P")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K4">
         <f>ROUND(J4*10/4,0)</f>
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="L4" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" t="s">
-        <v>193</v>
-      </c>
+      <c r="A5" s="53">
+        <v>5</v>
+      </c>
+      <c r="B5" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="C5" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D5" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53" t="s">
+        <v>193</v>
+      </c>
+      <c r="G5" s="54" t="s">
+        <v>194</v>
+      </c>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
       <c r="J5">
         <f>COUNTIF(E5:I5,"P")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K5">
         <f>ROUND(J5*10/4,0)</f>
-        <v>8</v>
+        <v>0</v>
+      </c>
+      <c r="L5" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:13" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>187</v>
+        <v>84</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>188</v>
+        <v>85</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
+      </c>
+      <c r="G6"/>
+      <c r="H6" t="s">
+        <v>193</v>
+      </c>
+      <c r="I6" t="s">
+        <v>193</v>
       </c>
       <c r="J6">
         <f>COUNTIF(E6:I6,"P")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <f>ROUND(J6*10/4,0)</f>
-        <v>8</v>
+        <v>0</v>
+      </c>
+      <c r="L6" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H7" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>22</v>
+        <v>22</v>
+      </c>
+      <c r="H7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" t="s">
+        <v>193</v>
       </c>
       <c r="J7">
         <f>COUNTIF(E7:I7,"P")</f>
@@ -4795,25 +4808,25 @@
         <f>ROUND(J7*10/4,0)</f>
         <v>8</v>
       </c>
+      <c r="L7" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="H8" t="s">
         <v>193</v>
@@ -4823,130 +4836,137 @@
       </c>
       <c r="J8">
         <f>COUNTIF(E8:I8,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <f>ROUND(J8*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="L8" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>14</v>
+        <v>187</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
+        <v>188</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H9" t="s">
-        <v>193</v>
-      </c>
-      <c r="I9" t="s">
+      <c r="F9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="7" t="s">
         <v>22</v>
       </c>
       <c r="J9">
         <f>COUNTIF(E9:I9,"P")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9">
         <f>ROUND(J9*10/4,0)</f>
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="L9" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H10" t="s">
-        <v>193</v>
-      </c>
-      <c r="I10" t="s">
+        <v>193</v>
+      </c>
+      <c r="G10" s="56"/>
+      <c r="H10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J10">
         <f>COUNTIF(E10:I10,"P")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10">
         <f>ROUND(J10*10/4,0)</f>
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="L10" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>132</v>
+        <v>34</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>191</v>
+        <v>35</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J11">
         <f>COUNTIF(E11:I11,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K11">
         <f>ROUND(J11*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="L11" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>140</v>
+        <v>108</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F12" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>193</v>
@@ -4956,32 +4976,37 @@
       </c>
       <c r="J12">
         <f>COUNTIF(E12:I12,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K12">
         <f>ROUND(J12*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="L12" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D13" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="57" t="s">
         <v>38</v>
       </c>
+      <c r="E13" s="57" t="s">
+        <v>22</v>
+      </c>
       <c r="F13" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="G13" s="56"/>
       <c r="H13" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>193</v>
@@ -4994,16 +5019,19 @@
         <f>ROUND(J13*10/4,0)</f>
         <v>3</v>
       </c>
+      <c r="L13" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>114</v>
+        <v>41</v>
       </c>
       <c r="D14" s="57" t="s">
         <v>38</v>
@@ -5028,22 +5056,22 @@
         <f>ROUND(J14*10/4,0)</f>
         <v>3</v>
       </c>
+      <c r="L14" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" s="57" t="s">
-        <v>22</v>
+        <v>50</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>193</v>
@@ -5056,11 +5084,14 @@
       </c>
       <c r="J15">
         <f>COUNTIF(E15:I15,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15">
         <f>ROUND(J15*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="L15" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
@@ -5096,23 +5127,23 @@
         <f>ROUND(J16*10/4,0)</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>56</v>
+        <v>189</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>57</v>
+        <v>190</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F17" s="7" t="s">
         <v>193</v>
       </c>
@@ -5124,31 +5155,37 @@
       </c>
       <c r="J17">
         <f>COUNTIF(E17:I17,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17">
         <f>ROUND(J17*10/4,0)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="L17" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>193</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>193</v>
@@ -5161,27 +5198,30 @@
         <f>ROUND(J18*10/4,0)</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>75</v>
+        <v>129</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>76</v>
+        <v>130</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="H19" t="s">
-        <v>193</v>
-      </c>
-      <c r="I19" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J19">
@@ -5192,89 +5232,98 @@
         <f>ROUND(J19*10/4,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="53">
-        <v>5</v>
-      </c>
-      <c r="B20" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="C20" s="53" t="s">
-        <v>185</v>
-      </c>
-      <c r="D20" s="53" t="s">
+      <c r="L19" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>24</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="53"/>
-      <c r="F20" s="53" t="s">
-        <v>193</v>
-      </c>
-      <c r="G20" s="54" t="s">
-        <v>194</v>
-      </c>
-      <c r="H20" s="54"/>
-      <c r="I20" s="54"/>
+      <c r="F20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>193</v>
+      </c>
       <c r="J20">
         <f>COUNTIF(E20:I20,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K20">
         <f>ROUND(J20*10/4,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="L20" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H21" t="s">
-        <v>193</v>
-      </c>
-      <c r="I21" t="s">
+      <c r="H21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J21">
         <f>COUNTIF(E21:I21,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21">
         <f>ROUND(J21*10/4,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+      <c r="L21" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>90</v>
+        <v>136</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H22" t="s">
-        <v>193</v>
-      </c>
-      <c r="I22" t="s">
+      <c r="H22" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J22">
@@ -5285,22 +5334,31 @@
         <f>ROUND(J22*10/4,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>34</v>
+        <v>139</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>35</v>
+        <v>140</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>195</v>
       </c>
       <c r="H23" s="7" t="s">
         <v>193</v>
@@ -5310,193 +5368,290 @@
       </c>
       <c r="J23">
         <f>COUNTIF(E23:I23,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K23">
         <f>ROUND(J23*10/4,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="L23" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
+        <v>3</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="C24" s="1" t="s">
-        <v>108</v>
+        <v>15</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>193</v>
+      <c r="F24" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" t="s">
+        <v>193</v>
+      </c>
+      <c r="I24" t="s">
+        <v>22</v>
       </c>
       <c r="J24">
         <f>COUNTIF(E24:I24,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K24">
         <f>ROUND(J24*10/4,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="L24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>49</v>
+        <v>202</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>50</v>
+        <v>203</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J25">
-        <f>COUNTIF(E25:I25,"P")</f>
-        <v>0</v>
-      </c>
-      <c r="K25">
-        <f>ROUND(J25*10/4,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+        <v>200</v>
+      </c>
+      <c r="F25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="L25" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J26">
-        <f>COUNTIF(E26:I26,"P")</f>
-        <v>0</v>
-      </c>
-      <c r="K26">
-        <f>ROUND(J26*10/4,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+        <v>200</v>
+      </c>
+      <c r="F26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="L26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>129</v>
+        <v>186</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>130</v>
+        <v>24</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
+      </c>
+      <c r="H27" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" t="s">
+        <v>22</v>
       </c>
       <c r="J27">
         <f>COUNTIF(E27:I27,"P")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K27">
         <f>ROUND(J27*10/4,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="L27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>136</v>
+        <v>104</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>137</v>
+        <v>105</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H28" s="7" t="s">
-        <v>193</v>
+      <c r="H28" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="J28">
         <f>COUNTIF(E28:I28,"P")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K28">
         <f>ROUND(J28*10/4,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="L28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
+        <v>15</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="D29" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29">
+        <f>COUNTIF(E29:I29,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K29">
+        <f>ROUND(J29*10/4,0)</f>
+        <v>10</v>
+      </c>
+      <c r="L29" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
+        <v>18</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J30">
+        <f>COUNTIF(E30:I30,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K30">
+        <f>ROUND(J30*10/4,0)</f>
+        <v>10</v>
+      </c>
+      <c r="L30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
+        <v>28</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="F31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+      <c r="L31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="D32" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E32" s="1">
         <f>COUNTIF(E2:E28,"P")</f>
-        <v>12</v>
-      </c>
-      <c r="F29" s="1">
+        <v>10</v>
+      </c>
+      <c r="F32" s="1">
         <f>COUNTIF(F2:F28,"P")</f>
-        <v>10</v>
-      </c>
-      <c r="H29" s="1">
+        <v>8</v>
+      </c>
+      <c r="H32" s="1">
         <f>COUNTIF(H2:H28,"P")</f>
-        <v>9</v>
-      </c>
-      <c r="I29" s="57">
+        <v>7</v>
+      </c>
+      <c r="I32" s="57">
         <f>COUNTIF(I2:I28,"P")</f>
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="L32" s="1">
+        <f>COUNTIF(L2:L31,"P")</f>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:K28">
-    <sortCondition descending="1" ref="K2:K28"/>
-    <sortCondition ref="B2:B28"/>
+  <sortState ref="A2:L31">
+    <sortCondition ref="L2:L31"/>
+    <sortCondition ref="B2:B31"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
agregado de acciones realizadas en clase en minuta
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="alumnos" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="203">
   <si>
     <t>Alumnos</t>
   </si>
@@ -616,9 +616,6 @@
   </si>
   <si>
     <t>prsentes</t>
-  </si>
-  <si>
-    <t>x</t>
   </si>
   <si>
     <t>nota</t>
@@ -4585,13 +4582,13 @@
         <v>196</v>
       </c>
       <c r="K1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="L1" s="52">
         <v>46177</v>
       </c>
-      <c r="M1">
-        <v>10</v>
+      <c r="M1" s="52">
+        <v>46184</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
@@ -4631,7 +4628,7 @@
         <v>193</v>
       </c>
       <c r="M2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -4667,6 +4664,9 @@
       <c r="L3" t="s">
         <v>193</v>
       </c>
+      <c r="M3" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -4702,6 +4702,9 @@
         <v>5</v>
       </c>
       <c r="L4" t="s">
+        <v>193</v>
+      </c>
+      <c r="M4" t="s">
         <v>193</v>
       </c>
     </row>
@@ -4738,6 +4741,9 @@
       <c r="L5" t="s">
         <v>193</v>
       </c>
+      <c r="M5" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="6" spans="1:13" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -4774,6 +4780,9 @@
       <c r="L6" t="s">
         <v>193</v>
       </c>
+      <c r="M6" s="54" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -4811,6 +4820,9 @@
       <c r="L7" t="s">
         <v>193</v>
       </c>
+      <c r="M7" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -4845,6 +4857,9 @@
       <c r="L8" t="s">
         <v>193</v>
       </c>
+      <c r="M8" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -4882,6 +4897,9 @@
       <c r="L9" t="s">
         <v>193</v>
       </c>
+      <c r="M9" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -4917,53 +4935,62 @@
       <c r="L10" t="s">
         <v>193</v>
       </c>
+      <c r="M10" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>34</v>
+        <v>104</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H11" s="7" t="s">
-        <v>193</v>
+      <c r="H11" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="J11">
         <f>COUNTIF(E11:I11,"P")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K11">
         <f>ROUND(J11*10/4,0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L11" t="s">
+        <v>22</v>
+      </c>
+      <c r="M11" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>107</v>
+        <v>34</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>108</v>
+        <v>35</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>193</v>
@@ -4985,22 +5012,22 @@
       <c r="L12" t="s">
         <v>193</v>
       </c>
+      <c r="M12" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D13" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E13" s="57" t="s">
-        <v>22</v>
+        <v>108</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>193</v>
@@ -5013,25 +5040,28 @@
       </c>
       <c r="J13">
         <f>COUNTIF(E13:I13,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13">
         <f>ROUND(J13*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L13" t="s">
+        <v>193</v>
+      </c>
+      <c r="M13" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>41</v>
+        <v>114</v>
       </c>
       <c r="D14" s="57" t="s">
         <v>38</v>
@@ -5059,19 +5089,25 @@
       <c r="L14" t="s">
         <v>193</v>
       </c>
+      <c r="M14" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>53</v>
+        <v>41</v>
+      </c>
+      <c r="D15" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>193</v>
@@ -5084,31 +5120,31 @@
       </c>
       <c r="J15">
         <f>COUNTIF(E15:I15,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15">
         <f>ROUND(J15*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L15" t="s">
+        <v>193</v>
+      </c>
+      <c r="M15" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>117</v>
+        <v>49</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>193</v>
@@ -5121,29 +5157,35 @@
       </c>
       <c r="J16">
         <f>COUNTIF(E16:I16,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16">
         <f>ROUND(J16*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L16" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M16" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>189</v>
+        <v>117</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>190</v>
+        <v>118</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="E17" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F17" s="7" t="s">
         <v>193</v>
       </c>
@@ -5155,32 +5197,32 @@
       </c>
       <c r="J17">
         <f>COUNTIF(E17:I17,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17">
         <f>ROUND(J17*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L17" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M17" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>56</v>
+        <v>189</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>57</v>
+        <v>190</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F18" s="7" t="s">
         <v>193</v>
       </c>
@@ -5192,28 +5234,34 @@
       </c>
       <c r="J18">
         <f>COUNTIF(E18:I18,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18">
         <f>ROUND(J18*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L18" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M18" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>129</v>
+        <v>56</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>130</v>
+        <v>57</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>193</v>
@@ -5226,65 +5274,71 @@
       </c>
       <c r="J19">
         <f>COUNTIF(E19:I19,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19">
         <f>ROUND(J19*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L19" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M19" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>191</v>
+        <v>130</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I20" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J20">
         <f>COUNTIF(E20:I20,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K20">
         <f>ROUND(J20*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L20" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M20" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>69</v>
+        <v>191</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>22</v>
@@ -5294,71 +5348,71 @@
       </c>
       <c r="J21">
         <f>COUNTIF(E21:I21,"P")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21">
         <f>ROUND(J21*10/4,0)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L21" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M21" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>136</v>
+        <v>64</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>137</v>
+        <v>69</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>193</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J22">
         <f>COUNTIF(E22:I22,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22">
         <f>ROUND(J22*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L22" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M22" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H23" s="7" t="s">
         <v>193</v>
@@ -5368,37 +5422,46 @@
       </c>
       <c r="J23">
         <f>COUNTIF(E23:I23,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K23">
         <f>ROUND(J23*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L23" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M23" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>15</v>
+        <v>140</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H24" t="s">
-        <v>193</v>
-      </c>
-      <c r="I24" t="s">
-        <v>22</v>
+      <c r="E24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>193</v>
       </c>
       <c r="J24">
         <f>COUNTIF(E24:I24,"P")</f>
@@ -5409,41 +5472,61 @@
         <v>5</v>
       </c>
       <c r="L24" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="M24" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
+        <v>3</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25" t="s">
+        <v>193</v>
+      </c>
+      <c r="I25" t="s">
+        <v>22</v>
+      </c>
+      <c r="J25">
+        <f>COUNTIF(E25:I25,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K25">
+        <f>ROUND(J25*10/4,0)</f>
+        <v>5</v>
+      </c>
+      <c r="L25" t="s">
+        <v>22</v>
+      </c>
+      <c r="M25" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
         <v>30</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B26" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="F25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="L25" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>29</v>
-      </c>
-      <c r="B26" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>200</v>
       </c>
       <c r="F26" s="7"/>
       <c r="H26" s="7"/>
@@ -5451,53 +5534,42 @@
       <c r="L26" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
+        <v>29</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="L27" t="s">
+        <v>22</v>
+      </c>
+      <c r="M27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
         <v>9</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H27" t="s">
-        <v>22</v>
-      </c>
-      <c r="I27" t="s">
-        <v>22</v>
-      </c>
-      <c r="J27">
-        <f>COUNTIF(E27:I27,"P")</f>
-        <v>4</v>
-      </c>
-      <c r="K27">
-        <f>ROUND(J27*10/4,0)</f>
-        <v>10</v>
-      </c>
-      <c r="L27" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>12</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>17</v>
@@ -5506,27 +5578,30 @@
         <v>22</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H28" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="I28" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" t="s">
         <v>22</v>
       </c>
       <c r="J28">
         <f>COUNTIF(E28:I28,"P")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K28">
         <f>ROUND(J28*10/4,0)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L28" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>15</v>
       </c>
@@ -5565,8 +5640,11 @@
       <c r="L29" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M29" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>18</v>
       </c>
@@ -5602,8 +5680,11 @@
       <c r="L30" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>28</v>
       </c>
@@ -5614,7 +5695,7 @@
         <v>188</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F31" s="7"/>
       <c r="H31" s="7"/>
@@ -5622,8 +5703,11 @@
       <c r="L31" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="D32" s="1" t="s">
         <v>192</v>
       </c>
@@ -5647,10 +5731,14 @@
         <f>COUNTIF(L2:L31,"P")</f>
         <v>8</v>
       </c>
+      <c r="M32" s="1">
+        <f>COUNTIF(M2:M31,"P")</f>
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:L31">
-    <sortCondition ref="L2:L31"/>
+  <sortState ref="A2:M31">
+    <sortCondition ref="M2:M31"/>
     <sortCondition ref="B2:B31"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>

</xml_diff>

<commit_message>
actualizacion de listado y agregado de minuta del 25-06-2026
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="207">
   <si>
     <t>Alumnos</t>
   </si>
@@ -634,6 +634,18 @@
   </si>
   <si>
     <t>Juan</t>
+  </si>
+  <si>
+    <t>Matorelli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lopez </t>
+  </si>
+  <si>
+    <t>Joaquin Alejandro</t>
+  </si>
+  <si>
+    <t>4A</t>
   </si>
 </sst>
 </file>
@@ -4538,19 +4550,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" customWidth="1"/>
-    <col min="8" max="10" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="1" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" hidden="1" customWidth="1"/>
+    <col min="8" max="10" width="11.5703125" hidden="1" customWidth="1"/>
+    <col min="11" max="12" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4590,8 +4603,14 @@
       <c r="M1" s="52">
         <v>46184</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N1" s="52">
+        <v>46191</v>
+      </c>
+      <c r="O1" s="52">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -4630,8 +4649,14 @@
       <c r="M2" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N2" t="s">
+        <v>193</v>
+      </c>
+      <c r="O2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -4667,8 +4692,14 @@
       <c r="M3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N3" t="s">
+        <v>193</v>
+      </c>
+      <c r="O3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>4</v>
       </c>
@@ -4707,8 +4738,14 @@
       <c r="M4" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N4" t="s">
+        <v>193</v>
+      </c>
+      <c r="O4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="53">
         <v>5</v>
       </c>
@@ -4744,8 +4781,14 @@
       <c r="M5" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="N5" t="s">
+        <v>193</v>
+      </c>
+      <c r="O5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>6</v>
       </c>
@@ -4783,8 +4826,14 @@
       <c r="M6" s="54" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N6" t="s">
+        <v>193</v>
+      </c>
+      <c r="O6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>7</v>
       </c>
@@ -4823,8 +4872,14 @@
       <c r="M7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N7" t="s">
+        <v>193</v>
+      </c>
+      <c r="O7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>8</v>
       </c>
@@ -4860,8 +4915,14 @@
       <c r="M8" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N8" t="s">
+        <v>193</v>
+      </c>
+      <c r="O8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>10</v>
       </c>
@@ -4900,8 +4961,14 @@
       <c r="M9" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N9" t="s">
+        <v>22</v>
+      </c>
+      <c r="O9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>11</v>
       </c>
@@ -4938,8 +5005,14 @@
       <c r="M10" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N10" t="s">
+        <v>193</v>
+      </c>
+      <c r="O10" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>12</v>
       </c>
@@ -4978,8 +5051,14 @@
       <c r="M11" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N11" t="s">
+        <v>193</v>
+      </c>
+      <c r="O11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>13</v>
       </c>
@@ -5015,8 +5094,14 @@
       <c r="M12" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N12" t="s">
+        <v>193</v>
+      </c>
+      <c r="O12" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>14</v>
       </c>
@@ -5052,56 +5137,71 @@
       <c r="M13" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N13" t="s">
+        <v>193</v>
+      </c>
+      <c r="O13" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D14" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" s="57" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>195</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="J14">
         <f>COUNTIF(E14:I14,"P")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K14">
         <f>ROUND(J14*10/4,0)</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L14" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="M14" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="N14" t="s">
+        <v>193</v>
+      </c>
+      <c r="O14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>41</v>
+        <v>114</v>
       </c>
       <c r="D15" s="57" t="s">
         <v>38</v>
@@ -5132,19 +5232,28 @@
       <c r="M15" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N15" t="s">
+        <v>193</v>
+      </c>
+      <c r="O15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>53</v>
+        <v>41</v>
+      </c>
+      <c r="D16" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>193</v>
@@ -5157,11 +5266,11 @@
       </c>
       <c r="J16">
         <f>COUNTIF(E16:I16,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16">
         <f>ROUND(J16*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L16" t="s">
         <v>193</v>
@@ -5169,22 +5278,25 @@
       <c r="M16" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N16" t="s">
+        <v>193</v>
+      </c>
+      <c r="O16" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>117</v>
+        <v>49</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>193</v>
@@ -5197,11 +5309,11 @@
       </c>
       <c r="J17">
         <f>COUNTIF(E17:I17,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17">
         <f>ROUND(J17*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L17" t="s">
         <v>193</v>
@@ -5209,20 +5321,29 @@
       <c r="M17" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N17" t="s">
+        <v>193</v>
+      </c>
+      <c r="O17" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>189</v>
+        <v>117</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>190</v>
+        <v>118</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="E18" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F18" s="7" t="s">
         <v>193</v>
       </c>
@@ -5234,11 +5355,11 @@
       </c>
       <c r="J18">
         <f>COUNTIF(E18:I18,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18">
         <f>ROUND(J18*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L18" t="s">
         <v>193</v>
@@ -5246,23 +5367,26 @@
       <c r="M18" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N18" t="s">
+        <v>193</v>
+      </c>
+      <c r="O18" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>56</v>
+        <v>189</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>57</v>
+        <v>190</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E19" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F19" s="7" t="s">
         <v>193</v>
       </c>
@@ -5274,11 +5398,11 @@
       </c>
       <c r="J19">
         <f>COUNTIF(E19:I19,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19">
         <f>ROUND(J19*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L19" t="s">
         <v>193</v>
@@ -5286,19 +5410,28 @@
       <c r="M19" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N19" t="s">
+        <v>193</v>
+      </c>
+      <c r="O19" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>129</v>
+        <v>56</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>130</v>
+        <v>57</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>193</v>
@@ -5311,11 +5444,11 @@
       </c>
       <c r="J20">
         <f>COUNTIF(E20:I20,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20">
         <f>ROUND(J20*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L20" t="s">
         <v>193</v>
@@ -5323,36 +5456,42 @@
       <c r="M20" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N20" t="s">
+        <v>193</v>
+      </c>
+      <c r="O20" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>191</v>
+        <v>130</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I21" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J21">
         <f>COUNTIF(E21:I21,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K21">
         <f>ROUND(J21*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L21" t="s">
         <v>193</v>
@@ -5360,22 +5499,28 @@
       <c r="M21" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N21" t="s">
+        <v>193</v>
+      </c>
+      <c r="O21" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>69</v>
+        <v>191</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="H22" s="7" t="s">
         <v>22</v>
@@ -5385,11 +5530,11 @@
       </c>
       <c r="J22">
         <f>COUNTIF(E22:I22,"P")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22">
         <f>ROUND(J22*10/4,0)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L22" t="s">
         <v>193</v>
@@ -5397,36 +5542,42 @@
       <c r="M22" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N22" t="s">
+        <v>193</v>
+      </c>
+      <c r="O22" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>136</v>
+        <v>64</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>137</v>
+        <v>69</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>193</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="I23" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J23">
         <f>COUNTIF(E23:I23,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23">
         <f>ROUND(J23*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L23" t="s">
         <v>193</v>
@@ -5434,28 +5585,28 @@
       <c r="M23" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N23" t="s">
+        <v>193</v>
+      </c>
+      <c r="O23" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H24" s="7" t="s">
         <v>193</v>
@@ -5465,11 +5616,11 @@
       </c>
       <c r="J24">
         <f>COUNTIF(E24:I24,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K24">
         <f>ROUND(J24*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L24" t="s">
         <v>193</v>
@@ -5477,28 +5628,40 @@
       <c r="M24" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N24" t="s">
+        <v>193</v>
+      </c>
+      <c r="O24" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>15</v>
+        <v>140</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H25" t="s">
-        <v>193</v>
-      </c>
-      <c r="I25" t="s">
-        <v>22</v>
+      <c r="E25" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>193</v>
       </c>
       <c r="J25">
         <f>COUNTIF(E25:I25,"P")</f>
@@ -5509,44 +5672,70 @@
         <v>5</v>
       </c>
       <c r="L25" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="M25" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="N25" t="s">
+        <v>193</v>
+      </c>
+      <c r="O25" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
+        <v>3</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" t="s">
+        <v>193</v>
+      </c>
+      <c r="I26" t="s">
+        <v>22</v>
+      </c>
+      <c r="J26">
+        <f>COUNTIF(E26:I26,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K26">
+        <f>ROUND(J26*10/4,0)</f>
+        <v>5</v>
+      </c>
+      <c r="L26" t="s">
+        <v>22</v>
+      </c>
+      <c r="M26" t="s">
+        <v>22</v>
+      </c>
+      <c r="N26" t="s">
+        <v>193</v>
+      </c>
+      <c r="O26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
         <v>30</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="F26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="L26" t="s">
-        <v>22</v>
-      </c>
-      <c r="M26" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>29</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>200</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>199</v>
@@ -5560,56 +5749,51 @@
       <c r="M27" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N27" t="s">
+        <v>22</v>
+      </c>
+      <c r="O27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
+        <v>29</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="L28" t="s">
+        <v>22</v>
+      </c>
+      <c r="M28" t="s">
+        <v>22</v>
+      </c>
+      <c r="N28" t="s">
+        <v>22</v>
+      </c>
+      <c r="O28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
         <v>9</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B29" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C29" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H28" t="s">
-        <v>22</v>
-      </c>
-      <c r="I28" t="s">
-        <v>22</v>
-      </c>
-      <c r="J28">
-        <f>COUNTIF(E28:I28,"P")</f>
-        <v>4</v>
-      </c>
-      <c r="K28">
-        <f>ROUND(J28*10/4,0)</f>
-        <v>10</v>
-      </c>
-      <c r="L28" t="s">
-        <v>22</v>
-      </c>
-      <c r="M28" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>15</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>17</v>
@@ -5620,13 +5804,10 @@
       <c r="F29" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G29" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="7" t="s">
+      <c r="H29" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" t="s">
         <v>22</v>
       </c>
       <c r="J29">
@@ -5643,103 +5824,172 @@
       <c r="M29" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N29" t="s">
+        <v>22</v>
+      </c>
+      <c r="O29" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
+        <v>32</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
+      <c r="O30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
         <v>18</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E30" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J30">
-        <f>COUNTIF(E30:I30,"P")</f>
+      <c r="E31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J31">
+        <f>COUNTIF(E31:I31,"P")</f>
         <v>4</v>
       </c>
-      <c r="K30">
-        <f>ROUND(J30*10/4,0)</f>
+      <c r="K31">
+        <f>ROUND(J31*10/4,0)</f>
         <v>10</v>
       </c>
-      <c r="L30" t="s">
-        <v>22</v>
-      </c>
-      <c r="M30" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A31" s="1">
+      <c r="L31" t="s">
+        <v>22</v>
+      </c>
+      <c r="M31" t="s">
+        <v>22</v>
+      </c>
+      <c r="N31" t="s">
+        <v>22</v>
+      </c>
+      <c r="O31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
         <v>28</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="F31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="L31" t="s">
-        <v>22</v>
-      </c>
-      <c r="M31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D32" s="1" t="s">
+      <c r="F32" s="7"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+      <c r="L32" t="s">
+        <v>22</v>
+      </c>
+      <c r="M32" t="s">
+        <v>22</v>
+      </c>
+      <c r="N32" t="s">
+        <v>22</v>
+      </c>
+      <c r="O32" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
+        <v>31</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
+      <c r="N33" t="s">
+        <v>22</v>
+      </c>
+      <c r="O33" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="D34" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E34" s="1">
         <f>COUNTIF(E2:E28,"P")</f>
         <v>10</v>
       </c>
-      <c r="F32" s="1">
+      <c r="F34" s="1">
         <f>COUNTIF(F2:F28,"P")</f>
         <v>8</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H34" s="1">
         <f>COUNTIF(H2:H28,"P")</f>
         <v>7</v>
       </c>
-      <c r="I32" s="57">
+      <c r="I34" s="57">
         <f>COUNTIF(I2:I28,"P")</f>
         <v>4</v>
       </c>
-      <c r="L32" s="1">
+      <c r="L34" s="1">
         <f>COUNTIF(L2:L31,"P")</f>
+        <v>7</v>
+      </c>
+      <c r="M34" s="1">
+        <f>COUNTIF(M2:M31,"P")</f>
+        <v>6</v>
+      </c>
+      <c r="N34" s="1">
+        <f>COUNTIF(N2:N32,"P")</f>
+        <v>6</v>
+      </c>
+      <c r="O34" s="1">
+        <f>COUNTIF(O2:O33,"P")</f>
         <v>8</v>
       </c>
-      <c r="M32" s="1">
-        <f>COUNTIF(M2:M31,"P")</f>
-        <v>7</v>
-      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:M31">
-    <sortCondition ref="M2:M31"/>
-    <sortCondition ref="B2:B31"/>
+  <sortState ref="A2:O33">
+    <sortCondition ref="O2:O33"/>
+    <sortCondition ref="B2:B33"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>